<commit_message>
Template: expand Anleitung tab with detailed field explanations (id/name/day_id/day_name/day_title, label, weight, warmup day_id matching)
</commit_message>
<xml_diff>
--- a/Program_Template.xlsx
+++ b/Program_Template.xlsx
@@ -116,12 +116,178 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t xml:space="preserve">=== FELDER IM DETAIL ===</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Program-Blatt:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  id    = interne Kurz-ID des GANZEN Programms. klein, keine Leerzeichen/Umlaute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Nie sichtbar, nur Technik. Pro Block eindeutig. Beispiel: mushin-p2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  name  = SICHTBARER Programmname auf der Startseite. Klartext mit Leerzeichen ok.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          Beispiel: Mushin - Phase 2: Hypertrophie</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  weeks = Anzahl Wochen (Zahl). Beispiel: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Exercises-Blatt - die drei Tag-Felder (in JEDER Zeile eines Tages GLEICH eintragen):</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  day_id    = stabile interne ID des Tages. klein, keine Leerzeichen/Umlaute.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              Verbindet alle Zeilen eines Tages UND verknuepft mit dem Warmups-Blatt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              &gt;&gt;&gt; EXAKT derselbe Wert muss im Warmups-Blatt stehen, sonst landet das</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              Warm-up im Nichts und es entsteht ein leerer Geister-Tag! &lt;&lt;&lt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              Beispiel: tag1   (nicht 'Tag 1' mit Leerzeichen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  day_name  = kurzes Label auf den Kacheln der Startseite. Kurz halten. Beispiel: Tag 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  day_title = volle Ueberschrift oben in der Logging-Ansicht. Darf beschreibend sein.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              Einheitlich bleiben (nicht mischen Tag1.. / Day3..). Beispiel: Tag 1 - Squat</t>
+        </is>
+      </c>
+    </row>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  label     = Uebungs-Label. Bei Supersaetzen pro Uebung UNTERSCHIEDLICH: 2a, 2b, 2c</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              (NICHT zweimal 2a! sonst sehen beide gleich aus)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  weight    = Richtgewicht kg. Bei Koerpergewicht-Uebungen LEER lassen (nicht 0).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  reps      = immer ausfuellen, auch bei Power-Uebungen (sonst zeigt die App leer).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Merksatz: day_id = fuer die App (technisch, einmal festlegen, nie aendern),</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          day_name = kurz fuer Kacheln, day_title = lang fuer die Kopfzeile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          day_id im Exercises- UND Warmups-Blatt muss identisch sein.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t xml:space="preserve">Danach konvertieren:  python tools/xlsx2program.py Program_Template.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="46">
+      <c r="A46" t="inlineStr">
         <is>
           <t xml:space="preserve">Das erzeugt program.json. Claude pusht es; auf dem Handy: Data -&gt; Reload program from file.</t>
         </is>

</xml_diff>

<commit_message>
feat(import): Excel per-week variation via week column (v1.17.0)
</commit_message>
<xml_diff>
--- a/Program_Template.xlsx
+++ b/Program_Template.xlsx
@@ -87,207 +87,228 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">3) Sheet 'Warmups' (optional): Warm-up &amp; Plyo-Block pro Tag. kind = warmup oder plyo.</t>
+          <t xml:space="preserve">   - week = leer/1 -&gt; Basis (gilt fuer ALLE Wochen). week = 2,3,... -&gt; nur diese Woche:</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   - Plyo-Einträge im Format 'Name :: schema', z.B. 'Reverse Pogos :: 20 reps · 30s · 2 Runden'.</t>
+          <t xml:space="preserve">       * gleiche Uebung + neue reps/rpe/weight = Ziel-Override pro Woche (Struktur bleibt).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">4) Übersprungener Tag (z.B. Taper-Ruhetag): in Warmups einen Eintrag mit der Notiz anlegen</t>
+          <t xml:space="preserve">       * neue/andere Uebungen in der Woche  = diese Woche wird eigenstaendig (eigene Struktur).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">   und in Exercises KEINE Zeilen für diesen day_id -&gt; wird als reiner Infotag angezeigt.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16"/>
+          <t xml:space="preserve">3) Sheet 'Warmups' (optional): Warm-up &amp; Plyo-Block pro Tag. kind = warmup oder plyo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   - Plyo-Einträge im Format 'Name :: schema', z.B. 'Reverse Pogos :: 20 reps · 30s · 2 Runden'.</t>
+        </is>
+      </c>
+    </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">=== FELDER IM DETAIL ===</t>
-        </is>
-      </c>
-    </row>
-    <row r="18"/>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Program-Blatt:</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">4) Übersprungener Tag (z.B. Taper-Ruhetag): in Warmups einen Eintrag mit der Notiz anlegen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   und in Exercises KEINE Zeilen für diesen day_id -&gt; wird als reiner Infotag angezeigt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">  id    = interne Kurz-ID des GANZEN Programms. klein, keine Leerzeichen/Umlaute.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">          Nie sichtbar, nur Technik. Pro Block eindeutig. Beispiel: mushin-p2</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">=== FELDER IM DETAIL ===</t>
+        </is>
+      </c>
+    </row>
+    <row r="21"/>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">  name  = SICHTBARER Programmname auf der Startseite. Klartext mit Leerzeichen ok.</t>
+          <t xml:space="preserve">Program-Blatt:</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">          Beispiel: Mushin - Phase 2: Hypertrophie</t>
+          <t xml:space="preserve">  id    = interne Kurz-ID des GANZEN Programms. klein, keine Leerzeichen/Umlaute.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  weeks = Anzahl Wochen (Zahl). Beispiel: 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="25"/>
+          <t xml:space="preserve">          Nie sichtbar, nur Technik. Pro Block eindeutig. Beispiel: mushin-p2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  name  = SICHTBARER Programmname auf der Startseite. Klartext mit Leerzeichen ok.</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Exercises-Blatt - die drei Tag-Felder (in JEDER Zeile eines Tages GLEICH eintragen):</t>
+          <t xml:space="preserve">          Beispiel: Mushin - Phase 2: Hypertrophie</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">  day_id    = stabile interne ID des Tages. klein, keine Leerzeichen/Umlaute.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">              Verbindet alle Zeilen eines Tages UND verknuepft mit dem Warmups-Blatt.</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">  weeks = Anzahl Wochen (Zahl). Beispiel: 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">              &gt;&gt;&gt; EXAKT derselbe Wert muss im Warmups-Blatt stehen, sonst landet das</t>
+          <t xml:space="preserve">Exercises-Blatt - die drei Tag-Felder (in JEDER Zeile eines Tages GLEICH eintragen):</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">              Warm-up im Nichts und es entsteht ein leerer Geister-Tag! &lt;&lt;&lt;</t>
+          <t xml:space="preserve">  day_id    = stabile interne ID des Tages. klein, keine Leerzeichen/Umlaute.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">              Beispiel: tag1   (nicht 'Tag 1' mit Leerzeichen)</t>
+          <t xml:space="preserve">              Verbindet alle Zeilen eines Tages UND verknuepft mit dem Warmups-Blatt.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">  day_name  = kurzes Label auf den Kacheln der Startseite. Kurz halten. Beispiel: Tag 1</t>
+          <t xml:space="preserve">              &gt;&gt;&gt; EXAKT derselbe Wert muss im Warmups-Blatt stehen, sonst landet das</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">  day_title = volle Ueberschrift oben in der Logging-Ansicht. Darf beschreibend sein.</t>
+          <t xml:space="preserve">              Warm-up im Nichts und es entsteht ein leerer Geister-Tag! &lt;&lt;&lt;</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">              Einheitlich bleiben (nicht mischen Tag1.. / Day3..). Beispiel: Tag 1 - Squat</t>
-        </is>
-      </c>
-    </row>
-    <row r="35"/>
+          <t xml:space="preserve">              Beispiel: tag1   (nicht 'Tag 1' mit Leerzeichen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  day_name  = kurzes Label auf den Kacheln der Startseite. Kurz halten. Beispiel: Tag 1</t>
+        </is>
+      </c>
+    </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">  label     = Uebungs-Label. Bei Supersaetzen pro Uebung UNTERSCHIEDLICH: 2a, 2b, 2c</t>
+          <t xml:space="preserve">  day_title = volle Ueberschrift oben in der Logging-Ansicht. Darf beschreibend sein.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">              (NICHT zweimal 2a! sonst sehen beide gleich aus)</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  weight    = Richtgewicht kg. Bei Koerpergewicht-Uebungen LEER lassen (nicht 0).</t>
-        </is>
-      </c>
-    </row>
+          <t xml:space="preserve">              Einheitlich bleiben (nicht mischen Tag1.. / Day3..). Beispiel: Tag 1 - Squat</t>
+        </is>
+      </c>
+    </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">  reps      = immer ausfuellen, auch bei Power-Uebungen (sonst zeigt die App leer).</t>
-        </is>
-      </c>
-    </row>
-    <row r="40"/>
+          <t xml:space="preserve">  label     = Uebungs-Label. Bei Supersaetzen pro Uebung UNTERSCHIEDLICH: 2a, 2b, 2c</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              (NICHT zweimal 2a! sonst sehen beide gleich aus)</t>
+        </is>
+      </c>
+    </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Merksatz: day_id = fuer die App (technisch, einmal festlegen, nie aendern),</t>
+          <t xml:space="preserve">  weight    = Richtgewicht kg. Bei Koerpergewicht-Uebungen LEER lassen (nicht 0).</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">          day_name = kurz fuer Kacheln, day_title = lang fuer die Kopfzeile.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">          day_id im Exercises- UND Warmups-Blatt muss identisch sein.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44"/>
+          <t xml:space="preserve">  reps      = immer ausfuellen, auch bei Power-Uebungen (sonst zeigt die App leer).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Merksatz: day_id = fuer die App (technisch, einmal festlegen, nie aendern),</t>
+        </is>
+      </c>
+    </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Danach konvertieren:  python tools/xlsx2program.py Program_Template.xlsx</t>
+          <t xml:space="preserve">          day_name = kurz fuer Kacheln, day_title = lang fuer die Kopfzeile.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">          day_id im Exercises- UND Warmups-Blatt muss identisch sein.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Danach konvertieren:  python tools/xlsx2program.py Program_Template.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
         <is>
           <t xml:space="preserve">Das erzeugt program.json. Claude pusht es; auf dem Handy: Data -&gt; Reload program from file.</t>
         </is>
@@ -414,6 +435,11 @@
           <t xml:space="preserve">max_lift_name</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">week</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -892,6 +918,98 @@
         <is>
           <t xml:space="preserve">x</t>
         </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lower</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lower</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Day 1 — Lower</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2a</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Back Squats</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="I12">
+        <v>8</v>
+      </c>
+      <c r="J12">
+        <v>102.5</v>
+      </c>
+      <c r="M12">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lower</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lower</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Day 1 — Lower</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2a</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Back Squats</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
+      <c r="I13">
+        <v>8.5</v>
+      </c>
+      <c r="J13">
+        <v>105</v>
+      </c>
+      <c r="M13">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>